<commit_message>
GA-RX/Kanal talebi eklendi; talep sayisi 22'ye cikti
Tablo B: Taslak 12 (BTK+Adalet Bak.) eklendi; matrise GA-RX/Kanal satiri;
Taslak 9/10/11 baslik stili + eksik muhatap satirlari; GA-1 dayanak duzeltmesi.
Analiz S6 talep tablosuna GA-RX/Kanal satiri (22 talep, yeniden numaralandi).
Envanter: ilgili satir kodu GA-RX/Kanal olarak hizalandi.
README, index.html: "21 talep" -> "22 talep". CHANGELOG guncellendi.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Amator_Telsizcilik_Tablo_A_Mevzuat_Envanteri_v1.0.xlsx
+++ b/Amator_Telsizcilik_Tablo_A_Mevzuat_Envanteri_v1.0.xlsx
@@ -3024,7 +3024,7 @@
     <row r="11" ht="90" customHeight="1" s="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>GA-RX</t>
+          <t>GA-RX/Kanal</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>dernek ve kulüpler ve kulüpler: Hafıza programlama disiplini konusunda üye bilgilendirmesi. Pratik öneri: Cihaz hafızası yalnızca amatör/yayıncılık bantlarını içermeli; askerî/güvenlik frekansları kaydedilmemeli. SDR preset dosyaları aynı dikkatle yönetilmeli.</t>
+          <t>Dernek ve kulüpler: Hafıza programlama disiplini konusunda üye bilgilendirmesi. Pratik öneri: Cihaz hafızası yalnızca amatör/yayıncılık bantlarını içermeli; askerî/güvenlik frekansları kaydedilmemeli. SDR preset dosyaları aynı dikkatle yönetilmeli. Ayrıca BTK ve Adalet Bakanlığı'na, kanal/tarama hafızasının olağan teknik özellik olduğu ve salt frekans kaydının başlı başına suç kastı göstermediği yönünde teknik açıklama/delil takdiri talebi (Tablo B Taslak 12).</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
GA-SK duzeltmesi: KEGM Yonetmeligi Md.7 birincil kaynak dogrulamasi
Md.7/1 (10 yillik bekletme) ve Md.7/2 (vefat/vesayette sartli varis/vasi
tahsisi) ayrimi netlestirildi. "Vesayet yolu tanimsiz/dayanaksiz" onculu
yanlisti - Md.7/2 bu yolu tanimliyor ama dar kapsamli (sure sonrasi akibet
belirsiz, esdeger belge sarti, ayni bolge ikamet sarti, KEGM takdiri).

Analiz (S3+S5), Envanter, Tablo B (Taslak 9) ve Oy Pusulasi'nda GA-SK
metni bu bulguya gore yeniden yazildi.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Amator_Telsizcilik_Tablo_A_Mevzuat_Envanteri_v1.0.xlsx
+++ b/Amator_Telsizcilik_Tablo_A_Mevzuat_Envanteri_v1.0.xlsx
@@ -3762,17 +3762,17 @@
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>Vefat/iptal sonrası 10 yıl pasif; in-memoriam vesayet</t>
+          <t>Md.7/2 vesayet mekanizması; süre sonrası akıbet ve eşdeğer belge şartı</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>KEGM Yönetmeliği, belge iptalinde (vefat dâhil) çağrı işaretini 10 yıl pasif tutar ve başkasına vermez/devredilemez. SK'nın resmî tanımı, 10 yıl sonrası akıbet ve aileye/kulübe 'in memoriam' vesayet yolu tanımsızdır. 'Babadan oğla geçme' fiilî bir talep olup hukuki dayanağı yoktur; bekleyeni almak isteyenler ile koruma/vesayet isteyenler arasında gerginlik vardır.</t>
+          <t>KEGM Yönetmeliği Md.7, vefatı 10 yıllık bekletme hükmünün (fıkra 1) kapsamı DIŞINDA tutar; fıkra 2 ayrı bir hüküm olarak, belgenin geçerlilik süresi içinde olmak, aynı bölgede ikamet etmek ve eşdeğer belgeye sahip olmak kaydıyla çağrı işaretinin varis/vasiye tahsis edilebileceğini düzenler. Yani 'vesayet yolu tanımsız/hukuki dayanaksız' algısı isabetli değildir; ancak mekanizma dardır: süre sonrası akıbet belirsiz, belgesiz aile üyeleri kapsam dışı, tahsis KEGM takdirinde.</t>
         </is>
       </c>
       <c r="E25" s="22" t="inlineStr">
         <is>
-          <t>KEGM Sınav ve Belgelendirme Yönetmeliği (RG 27482): belge iptali sonrası çağrı işareti 10 yıl yeniden tahsis edilmez; devredilemez.</t>
+          <t>KEGM Sınav ve Belgelendirme Yönetmeliği (RG 27482) Md.7/1 (10 yıl bekletme; vefat hariç) ve Md.7/2 (vefat/vesayette şartlı varis/vasi tahsisi).</t>
         </is>
       </c>
       <c r="F25" s="22" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="H25" s="22" t="inlineStr">
         <is>
-          <t>KEGM'den: (1) SK ve çağrı işareti yaşam döngüsünün tanımlanması; (2) bekletme süresinin (koru/uzat/kısalt/kaldır) ve vesayetin (devredilemez / şartlı aile-kulüp / süre sonu serbest / kalıcı anıt) usule bağlanması.</t>
+          <t>KEGM'den: (1) Md.7/2'nin belge süresi sonrası akıbetinin netleştirilmesi; (2) 'eşdeğer belge sahibi olma' şartının esnetilip esnetilemeyeceğinin değerlendirilmesi; (3) mekanizmanın topluluğa rehberle duyurulması.</t>
         </is>
       </c>
       <c r="I25" s="22" t="inlineStr">

</xml_diff>